<commit_message>
IV: lagged own price only (F=65 pre-COVID, F=99 full); drop bandwidth (Hansen J rejects); clean 3-row table; add Stock-Yogo bib entry
</commit_message>
<xml_diff>
--- a/results/regression_output/robustness/iv_results.xlsx
+++ b/results/regression_output/robustness/iv_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,65 +429,80 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>instruments</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>eu_elasticity</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>eu_se</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>eu_pval</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>eap_elasticity</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>eap_se</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>eap_pval</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>first_stage_f</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>first_stage_r2</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>hansen_j</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>hansen_p</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
         <is>
           <t>n_obs</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>price_x_covid_coef</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>price_x_covid_pval</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>price_x_eap_x_covid_coef</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>price_x_eap_x_covid_pval</t>
         </is>
@@ -502,122 +517,143 @@
       <c r="B2" t="b">
         <v>0</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
         <v>-0.1012746800182213</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>0.05275385897832809</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>0.05591911331221877</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>-0.5950760110920711</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>0.06080434296142238</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="n">
-        <v>330</v>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
+      <c r="N2" t="n">
+        <v>330</v>
+      </c>
       <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pre-COVID 2SLS</t>
+          <t>Pre-COVID: Lagged price</t>
         </is>
       </c>
       <c r="B3" t="b">
         <v>0</v>
       </c>
-      <c r="C3" t="n">
-        <v>-6.129399221376843</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>log_fixed_broad_price_lag1</t>
+        </is>
       </c>
       <c r="D3" t="n">
-        <v>51.78125315876899</v>
+        <v>-0.1721922546719625</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9057736951453184</v>
+        <v>0.09656309812222548</v>
       </c>
       <c r="F3" t="n">
-        <v>3.02574206525378</v>
+        <v>0.07455217163957761</v>
       </c>
       <c r="G3" t="n">
-        <v>10.08923261627137</v>
+        <v>-0.6150212572222991</v>
       </c>
       <c r="H3" t="n">
-        <v>0.7642548554327562</v>
+        <v>0.09106189823196463</v>
       </c>
       <c r="I3" t="n">
-        <v>0.4316893650883381</v>
+        <v>1.439404151426515e-11</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1861561020253039</v>
+        <v>65.06569103792789</v>
       </c>
       <c r="K3" t="n">
-        <v>330</v>
+        <v>0.4625010449662337</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="n">
+        <v>297</v>
+      </c>
       <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Full Sample 2SLS (COVID interactions)</t>
+          <t>Full sample: Lagged price</t>
         </is>
       </c>
       <c r="B4" t="b">
         <v>1</v>
       </c>
-      <c r="C4" t="n">
-        <v>-0.1708592398462737</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>log_fixed_broad_price_lag1</t>
+        </is>
       </c>
       <c r="D4" t="n">
-        <v>0.2386243575105937</v>
+        <v>-0.1925284570386452</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4739804812444774</v>
+        <v>0.05815399812019782</v>
       </c>
       <c r="F4" t="n">
-        <v>0.122935203770118</v>
+        <v>0.0009307427056890472</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1420502254928952</v>
+        <v>-0.339664543885963</v>
       </c>
       <c r="H4" t="n">
-        <v>0.386800205650897</v>
+        <v>0.08836257030983047</v>
       </c>
       <c r="I4" t="n">
-        <v>17.38250936332875</v>
+        <v>0.000121051575506792</v>
       </c>
       <c r="J4" t="n">
-        <v>0.3317244265897522</v>
+        <v>98.78290633720628</v>
       </c>
       <c r="K4" t="n">
-        <v>495</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.5284022038854497</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.164276927010556</v>
-      </c>
+        <v>0.6003835475632878</v>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>0.1168091962607301</v>
+        <v>462</v>
       </c>
       <c r="O4" t="n">
-        <v>0.4031358599695054</v>
+        <v>0.2562866085119027</v>
+      </c>
+      <c r="P4" t="n">
+        <v>8.730949052626613e-07</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.09637987175066023</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.003670077479816181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>